<commit_message>
Mettre à jour le calculateur de tarification CursAudit vers la version 1 (grille par tranches de pages)
</commit_message>
<xml_diff>
--- a/docs/pricing/cursaudit-calculateur-tarification.xlsx
+++ b/docs/pricing/cursaudit-calculateur-tarification.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40b6a5b8edd2a2a5/Bureau/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7B0B9670-820B-440D-8E9E-BBDB62319605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB133F92-E9AB-4B22-AA78-6430C6DBF0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,8 @@
     <sheet name="Scénarios" sheetId="3" r:id="rId3"/>
     <sheet name="Grille dimensions" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="109">
   <si>
     <t>CURSAUDIT — CALCULATEUR DE TARIFICATION</t>
   </si>
@@ -330,13 +331,46 @@
   </si>
   <si>
     <t>Marge bénéficiaire brute</t>
+  </si>
+  <si>
+    <t>20-29</t>
+  </si>
+  <si>
+    <t>30-39</t>
+  </si>
+  <si>
+    <t>50-99</t>
+  </si>
+  <si>
+    <t>10-19</t>
+  </si>
+  <si>
+    <t>39-49</t>
+  </si>
+  <si>
+    <t>moyenne</t>
+  </si>
+  <si>
+    <t>&lt;10 minimum</t>
+  </si>
+  <si>
+    <t>100-149</t>
+  </si>
+  <si>
+    <t>150-249</t>
+  </si>
+  <si>
+    <t>150-250</t>
+  </si>
+  <si>
+    <t>&gt;250</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.000\ \€"/>
     <numFmt numFmtId="165" formatCode="0.00\ \€"/>
@@ -344,8 +378,9 @@
     <numFmt numFmtId="167" formatCode="0.0\x"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
     <numFmt numFmtId="169" formatCode="0.00\x"/>
+    <numFmt numFmtId="170" formatCode="0\ \x"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -389,8 +424,12 @@
       <sz val="11"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Carlito"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -427,8 +466,14 @@
         <fgColor rgb="FFFFFDF0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -436,12 +481,123 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -491,17 +647,119 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="17" fontId="3" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -897,78 +1155,78 @@
           <c:invertIfNegative val="1"/>
           <c:cat>
             <c:numRef>
-              <c:f>Scénarios!$A$2:$A$11</c:f>
+              <c:f>Scénarios!$B$10:$B$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>50</c:v>
+                  <c:v>75</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>100</c:v>
+                  <c:v>75</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>150</c:v>
+                  <c:v>125</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>250</c:v>
+                  <c:v>125</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>150</c:v>
+                  <c:v>125</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>150</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>150</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>150</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>150</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>250</c:v>
+                  <c:v>300</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Scénarios!$I$2:$I$11</c:f>
+              <c:f>Scénarios!$J$10:$J$19</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.00\ \€</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>25.961249999999996</c:v>
+                  <c:v>35.491875</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>45.022499999999994</c:v>
+                  <c:v>60.509765625</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>64.083749999999995</c:v>
+                  <c:v>54.553124999999994</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>102.20624999999998</c:v>
+                  <c:v>96.249609374999991</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>170.55937499999999</c:v>
+                  <c:v>146.73281249999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>313.51874999999995</c:v>
+                  <c:v>408.82499999999987</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>470.77406250000001</c:v>
+                  <c:v>618.49874999999986</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>570.84562499999993</c:v>
+                  <c:v>751.92749999999978</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>699.50906250000003</c:v>
+                  <c:v>923.47874999999976</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1434.310546875</c:v>
+                  <c:v>1371.4181250000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1669,15 +1927,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
+      <xdr:col>21</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1913,14 +2171,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="18">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -1928,14 +2186,14 @@
       <c r="K1" s="1"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -1956,16 +2214,16 @@
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="1:11" ht="15">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25" t="s">
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
+      <c r="D4" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
+      <c r="E4" s="59"/>
+      <c r="F4" s="59"/>
       <c r="G4" s="1">
         <v>2</v>
       </c>
@@ -1997,15 +2255,15 @@
       <c r="F5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="20">
+      <c r="G5" s="18">
         <f>+G7-G6</f>
         <v>117.693515625</v>
       </c>
-      <c r="H5" s="20">
+      <c r="H5" s="18">
         <f>+H7-H6</f>
         <v>235.38703124999998</v>
       </c>
-      <c r="I5" s="20">
+      <c r="I5" s="18">
         <f>+I7-I6</f>
         <v>353.08054687499998</v>
       </c>
@@ -2031,16 +2289,16 @@
       <c r="F6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="19">
+      <c r="G6" s="17">
         <f>+$E$16</f>
         <v>117.693515625</v>
       </c>
-      <c r="H6" s="19">
-        <f t="shared" ref="H6:I6" si="0">+$E$16</f>
+      <c r="H6" s="17">
+        <f>+$E$16</f>
         <v>117.693515625</v>
       </c>
-      <c r="I6" s="19">
-        <f t="shared" si="0"/>
+      <c r="I6" s="17">
+        <f>+$E$16</f>
         <v>117.693515625</v>
       </c>
       <c r="J6" s="1"/>
@@ -2065,15 +2323,15 @@
       <c r="F7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="20">
+      <c r="G7" s="18">
         <f>+G6*G4</f>
         <v>235.38703125000001</v>
       </c>
-      <c r="H7" s="20">
+      <c r="H7" s="18">
         <f>+H6*H4</f>
         <v>353.08054687499998</v>
       </c>
-      <c r="I7" s="20">
+      <c r="I7" s="18">
         <f>+I6*I4</f>
         <v>470.77406250000001</v>
       </c>
@@ -2138,16 +2396,16 @@
       <c r="K10" s="1"/>
     </row>
     <row r="11" spans="1:11" ht="15">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="59" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25" t="s">
+      <c r="B11" s="59"/>
+      <c r="C11" s="59"/>
+      <c r="D11" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
+      <c r="E11" s="59"/>
+      <c r="F11" s="59"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
@@ -2351,14 +2609,14 @@
       <c r="K20" s="1"/>
     </row>
     <row r="21" spans="1:11" ht="15">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="55" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
+      <c r="B21" s="55"/>
+      <c r="C21" s="55"/>
+      <c r="D21" s="55"/>
+      <c r="E21" s="55"/>
+      <c r="F21" s="55"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
@@ -2366,14 +2624,14 @@
       <c r="K21" s="1"/>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="56" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
+      <c r="B22" s="56"/>
+      <c r="C22" s="56"/>
+      <c r="D22" s="56"/>
+      <c r="E22" s="56"/>
+      <c r="F22" s="56"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
@@ -2381,14 +2639,14 @@
       <c r="K22" s="1"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="56" t="s">
         <v>39</v>
       </c>
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
+      <c r="B23" s="56"/>
+      <c r="C23" s="56"/>
+      <c r="D23" s="56"/>
+      <c r="E23" s="56"/>
+      <c r="F23" s="56"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
@@ -3058,713 +3316,1120 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="1" max="1" width="12.375" style="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" style="20" customWidth="1"/>
+    <col min="3" max="3" width="11.25" style="20" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.375" style="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.375" style="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13" style="20" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5" style="20" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.75" style="20" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.25" style="20" bestFit="1" customWidth="1"/>
+    <col min="10" max="12" width="12.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:12" ht="15.75" thickBot="1">
+      <c r="A1" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="22" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="37" t="s">
         <v>75</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="38" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="17">
-        <v>50</v>
-      </c>
-      <c r="B2" s="17">
+    <row r="2" spans="1:12" ht="30">
+      <c r="A2" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="22">
+        <v>10</v>
+      </c>
+      <c r="C2" s="22">
         <v>8</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="D2" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="E2" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="E2" s="18">
+      <c r="F2" s="49">
+        <v>2</v>
+      </c>
+      <c r="G2" s="23">
+        <f>B2*Calculateur!$B$6*Calculateur!$B$12*(C2/Calculateur!$B$13)*IF(D2="1 IA",1,IF(D2="2 IA",1.55,IF(D2="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>1.105</v>
+      </c>
+      <c r="H2" s="23">
+        <f>G2+IF(E2="Aucun",0,IF(E2="Synthèse courte",2,6))</f>
+        <v>3.105</v>
+      </c>
+      <c r="I2" s="23">
+        <f>H2*(1+Calculateur!$E$6/100)</f>
+        <v>3.5707499999999999</v>
+      </c>
+      <c r="J2" s="24">
+        <f>I2*F2*(1-Calculateur!$E$8/100)</f>
+        <v>7.1414999999999997</v>
+      </c>
+      <c r="K2" s="24">
+        <f>J2*Calculateur!$E$7/100</f>
+        <v>1.4997149999999999</v>
+      </c>
+      <c r="L2" s="25">
+        <f>J2+K2</f>
+        <v>8.641214999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="30">
+      <c r="A3" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" s="3">
+        <v>15</v>
+      </c>
+      <c r="C3" s="3">
+        <v>8</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" s="50">
         <v>3</v>
       </c>
-      <c r="F2" s="19">
-        <f>A2*Calculateur!$B$6*Calculateur!$B$12*(B2/Calculateur!$B$13)*IF(C2="1 IA",1,IF(C2="2 IA",1.55,IF(C2="2 IA + confrontation ciblée",1.9,2.35)))</f>
-        <v>5.5249999999999995</v>
-      </c>
-      <c r="G2" s="19">
-        <f t="shared" ref="G2:G11" si="0">F2+IF(D2="Aucun",0,IF(D2="Synthèse courte",2,6))</f>
-        <v>7.5249999999999995</v>
-      </c>
-      <c r="H2" s="19">
-        <f>G2*(1+Calculateur!$E$6/100)</f>
-        <v>8.6537499999999987</v>
-      </c>
-      <c r="I2" s="19">
-        <f>H2*E2*(1-Calculateur!$E$8/100)</f>
-        <v>25.961249999999996</v>
-      </c>
-      <c r="J2" s="19">
-        <f>I2*Calculateur!$E$7/100</f>
-        <v>5.4518624999999998</v>
-      </c>
-      <c r="K2" s="19">
-        <f t="shared" ref="K2:K11" si="1">I2+J2</f>
-        <v>31.413112499999997</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="17">
+      <c r="G3" s="27">
+        <f>B3*Calculateur!$B$6*Calculateur!$B$12*(C3/Calculateur!$B$13)*IF(D3="1 IA",1,IF(D3="2 IA",1.55,IF(D3="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>1.6575</v>
+      </c>
+      <c r="H3" s="27">
+        <f>G3+IF(E3="Aucun",0,IF(E3="Synthèse courte",2,6))</f>
+        <v>3.6574999999999998</v>
+      </c>
+      <c r="I3" s="27">
+        <f>H3*(1+Calculateur!$E$6/100)</f>
+        <v>4.2061249999999992</v>
+      </c>
+      <c r="J3" s="17">
+        <f>I3*F3*(1-Calculateur!$E$8/100)</f>
+        <v>12.618374999999997</v>
+      </c>
+      <c r="K3" s="17">
+        <f>J3*Calculateur!$E$7/100</f>
+        <v>2.649858749999999</v>
+      </c>
+      <c r="L3" s="28">
+        <f>J3+K3</f>
+        <v>15.268233749999997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="30">
+      <c r="A4" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" s="30">
+        <v>25</v>
+      </c>
+      <c r="C4" s="3">
+        <v>8</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" s="50">
+        <v>3</v>
+      </c>
+      <c r="G4" s="27">
+        <f>B4*Calculateur!$B$6*Calculateur!$B$12*(C4/Calculateur!$B$13)*IF(D4="1 IA",1,IF(D4="2 IA",1.55,IF(D4="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>2.7624999999999997</v>
+      </c>
+      <c r="H4" s="27">
+        <f>G4+IF(E4="Aucun",0,IF(E4="Synthèse courte",2,6))</f>
+        <v>4.7624999999999993</v>
+      </c>
+      <c r="I4" s="27">
+        <f>H4*(1+Calculateur!$E$6/100)</f>
+        <v>5.4768749999999988</v>
+      </c>
+      <c r="J4" s="17">
+        <f>I4*F4*(1-Calculateur!$E$8/100)</f>
+        <v>16.430624999999996</v>
+      </c>
+      <c r="K4" s="17">
+        <f>J4*Calculateur!$E$7/100</f>
+        <v>3.4504312499999994</v>
+      </c>
+      <c r="L4" s="28">
+        <f>J4+K4</f>
+        <v>19.881056249999993</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="15.75" customHeight="1">
+      <c r="A5" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="30">
+        <v>25</v>
+      </c>
+      <c r="C5" s="3">
+        <v>15</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="50">
+        <v>3</v>
+      </c>
+      <c r="G5" s="27">
+        <f>B5*Calculateur!$B$6*Calculateur!$B$12*(C5/Calculateur!$B$13)*IF(D5="1 IA",1,IF(D5="2 IA",1.55,IF(D5="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>5.1796874999999991</v>
+      </c>
+      <c r="H5" s="27">
+        <f>G5+IF(E5="Aucun",0,IF(E5="Synthèse courte",2,6))</f>
+        <v>7.1796874999999991</v>
+      </c>
+      <c r="I5" s="27">
+        <f>H5*(1+Calculateur!$E$6/100)</f>
+        <v>8.2566406249999975</v>
+      </c>
+      <c r="J5" s="17">
+        <f>I5*F5*(1-Calculateur!$E$8/100)</f>
+        <v>24.769921874999994</v>
+      </c>
+      <c r="K5" s="17">
+        <f>J5*Calculateur!$E$7/100</f>
+        <v>5.2016835937499994</v>
+      </c>
+      <c r="L5" s="28">
+        <f>J5+K5</f>
+        <v>29.971605468749992</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="15.75" customHeight="1">
+      <c r="A6" s="31" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6" s="3">
+        <v>35</v>
+      </c>
+      <c r="C6" s="3">
+        <v>8</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" s="50">
+        <v>3</v>
+      </c>
+      <c r="G6" s="27">
+        <f>B6*Calculateur!$B$6*Calculateur!$B$12*(C6/Calculateur!$B$13)*IF(D6="1 IA",1,IF(D6="2 IA",1.55,IF(D6="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>3.8674999999999997</v>
+      </c>
+      <c r="H6" s="27">
+        <f t="shared" ref="H6:H11" si="0">G6+IF(E6="Aucun",0,IF(E6="Synthèse courte",2,6))</f>
+        <v>5.8674999999999997</v>
+      </c>
+      <c r="I6" s="27">
+        <f>H6*(1+Calculateur!$E$6/100)</f>
+        <v>6.7476249999999993</v>
+      </c>
+      <c r="J6" s="17">
+        <f>I6*F6*(1-Calculateur!$E$8/100)</f>
+        <v>20.242874999999998</v>
+      </c>
+      <c r="K6" s="17">
+        <f>J6*Calculateur!$E$7/100</f>
+        <v>4.2510037499999997</v>
+      </c>
+      <c r="L6" s="28">
+        <f t="shared" ref="L6:L11" si="1">J6+K6</f>
+        <v>24.493878749999997</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="15.75" customHeight="1">
+      <c r="A7" s="31" t="s">
+        <v>99</v>
+      </c>
+      <c r="B7" s="3">
+        <v>35</v>
+      </c>
+      <c r="C7" s="3">
+        <v>15</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" s="50">
+        <v>3</v>
+      </c>
+      <c r="G7" s="27">
+        <f>B7*Calculateur!$B$6*Calculateur!$B$12*(C7/Calculateur!$B$13)*IF(D7="1 IA",1,IF(D7="2 IA",1.55,IF(D7="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>7.2515624999999995</v>
+      </c>
+      <c r="H7" s="27">
+        <f t="shared" si="0"/>
+        <v>9.2515624999999986</v>
+      </c>
+      <c r="I7" s="27">
+        <f>H7*(1+Calculateur!$E$6/100)</f>
+        <v>10.639296874999998</v>
+      </c>
+      <c r="J7" s="17">
+        <f>I7*F7*(1-Calculateur!$E$8/100)</f>
+        <v>31.917890624999991</v>
+      </c>
+      <c r="K7" s="17">
+        <f>J7*Calculateur!$E$7/100</f>
+        <v>6.7027570312499982</v>
+      </c>
+      <c r="L7" s="28">
+        <f t="shared" si="1"/>
+        <v>38.620647656249986</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="15.75" customHeight="1">
+      <c r="A8" s="31" t="s">
+        <v>102</v>
+      </c>
+      <c r="B8" s="3">
+        <v>45</v>
+      </c>
+      <c r="C8" s="3">
+        <v>8</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F8" s="50">
+        <v>3</v>
+      </c>
+      <c r="G8" s="27">
+        <f>B8*Calculateur!$B$6*Calculateur!$B$12*(C8/Calculateur!$B$13)*IF(D8="1 IA",1,IF(D8="2 IA",1.55,IF(D8="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>4.9725000000000001</v>
+      </c>
+      <c r="H8" s="27">
+        <f t="shared" si="0"/>
+        <v>6.9725000000000001</v>
+      </c>
+      <c r="I8" s="27">
+        <f>H8*(1+Calculateur!$E$6/100)</f>
+        <v>8.0183749999999989</v>
+      </c>
+      <c r="J8" s="17">
+        <f>I8*F8*(1-Calculateur!$E$8/100)</f>
+        <v>24.055124999999997</v>
+      </c>
+      <c r="K8" s="17">
+        <f>J8*Calculateur!$E$7/100</f>
+        <v>5.0515762499999992</v>
+      </c>
+      <c r="L8" s="28">
+        <f t="shared" si="1"/>
+        <v>29.106701249999997</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A9" s="32" t="s">
+        <v>102</v>
+      </c>
+      <c r="B9" s="33">
+        <v>45</v>
+      </c>
+      <c r="C9" s="33">
+        <v>15</v>
+      </c>
+      <c r="D9" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" s="51">
+        <v>3</v>
+      </c>
+      <c r="G9" s="34">
+        <f>B9*Calculateur!$B$6*Calculateur!$B$12*(C9/Calculateur!$B$13)*IF(D9="1 IA",1,IF(D9="2 IA",1.55,IF(D9="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>9.3234375000000007</v>
+      </c>
+      <c r="H9" s="34">
+        <f t="shared" si="0"/>
+        <v>11.323437500000001</v>
+      </c>
+      <c r="I9" s="34">
+        <f>H9*(1+Calculateur!$E$6/100)</f>
+        <v>13.021953125</v>
+      </c>
+      <c r="J9" s="35">
+        <f>I9*F9*(1-Calculateur!$E$8/100)</f>
+        <v>39.065859375000002</v>
+      </c>
+      <c r="K9" s="35">
+        <f>J9*Calculateur!$E$7/100</f>
+        <v>8.2038304687500005</v>
+      </c>
+      <c r="L9" s="36">
+        <f t="shared" si="1"/>
+        <v>47.269689843750001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" s="39" t="s">
         <v>100</v>
       </c>
-      <c r="B3" s="17">
+      <c r="B10" s="40">
+        <v>75</v>
+      </c>
+      <c r="C10" s="40">
         <v>8</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="D10" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="E10" s="40" t="s">
         <v>59</v>
       </c>
-      <c r="E3" s="18">
+      <c r="F10" s="52">
         <v>3</v>
       </c>
-      <c r="F3" s="19">
-        <f>A3*Calculateur!$B$6*Calculateur!$B$12*(B3/Calculateur!$B$13)*IF(C3="1 IA",1,IF(C3="2 IA",1.55,IF(C3="2 IA + confrontation ciblée",1.9,2.35)))</f>
-        <v>11.049999999999999</v>
-      </c>
-      <c r="G3" s="19">
+      <c r="G10" s="27">
+        <f>B10*Calculateur!$B$6*Calculateur!$B$12*(C10/Calculateur!$B$13)*IF(D10="1 IA",1,IF(D10="2 IA",1.55,IF(D10="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>8.2874999999999996</v>
+      </c>
+      <c r="H10" s="27">
         <f t="shared" si="0"/>
-        <v>13.049999999999999</v>
-      </c>
-      <c r="H3" s="19">
-        <f>G3*(1+Calculateur!$E$6/100)</f>
-        <v>15.007499999999997</v>
-      </c>
-      <c r="I3" s="19">
-        <f>H3*E3*(1-Calculateur!$E$8/100)</f>
-        <v>45.022499999999994</v>
-      </c>
-      <c r="J3" s="19">
-        <f>I3*Calculateur!$E$7/100</f>
-        <v>9.454724999999998</v>
-      </c>
-      <c r="K3" s="19">
+        <v>10.2875</v>
+      </c>
+      <c r="I10" s="27">
+        <f>H10*(1+Calculateur!$E$6/100)</f>
+        <v>11.830625</v>
+      </c>
+      <c r="J10" s="17">
+        <f>I10*F10*(1-Calculateur!$E$8/100)</f>
+        <v>35.491875</v>
+      </c>
+      <c r="K10" s="17">
+        <f>J10*Calculateur!$E$7/100</f>
+        <v>7.4532937500000003</v>
+      </c>
+      <c r="L10" s="28">
         <f t="shared" si="1"/>
-        <v>54.47722499999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
-      <c r="A4" s="17">
-        <v>150</v>
-      </c>
-      <c r="B4" s="17">
+        <v>42.945168750000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" s="39" t="s">
+        <v>100</v>
+      </c>
+      <c r="B11" s="40">
+        <v>75</v>
+      </c>
+      <c r="C11" s="40">
+        <v>15</v>
+      </c>
+      <c r="D11" s="40" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="F11" s="52">
+        <v>3</v>
+      </c>
+      <c r="G11" s="27">
+        <f>B11*Calculateur!$B$6*Calculateur!$B$12*(C11/Calculateur!$B$13)*IF(D11="1 IA",1,IF(D11="2 IA",1.55,IF(D11="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>15.5390625</v>
+      </c>
+      <c r="H11" s="27">
+        <f t="shared" si="0"/>
+        <v>17.5390625</v>
+      </c>
+      <c r="I11" s="27">
+        <f>H11*(1+Calculateur!$E$6/100)</f>
+        <v>20.169921875</v>
+      </c>
+      <c r="J11" s="17">
+        <f>I11*F11*(1-Calculateur!$E$8/100)</f>
+        <v>60.509765625</v>
+      </c>
+      <c r="K11" s="17">
+        <f>J11*Calculateur!$E$7/100</f>
+        <v>12.70705078125</v>
+      </c>
+      <c r="L11" s="28">
+        <f t="shared" si="1"/>
+        <v>73.216816406250004</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" s="41" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" s="40">
+        <v>125</v>
+      </c>
+      <c r="C12" s="40">
         <v>8</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="D12" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="E12" s="40" t="s">
         <v>59</v>
       </c>
-      <c r="E4" s="18">
+      <c r="F12" s="52">
         <v>3</v>
       </c>
-      <c r="F4" s="19">
-        <f>A4*Calculateur!$B$6*Calculateur!$B$12*(B4/Calculateur!$B$13)*IF(C4="1 IA",1,IF(C4="2 IA",1.55,IF(C4="2 IA + confrontation ciblée",1.9,2.35)))</f>
-        <v>16.574999999999999</v>
-      </c>
-      <c r="G4" s="19">
-        <f t="shared" si="0"/>
-        <v>18.574999999999999</v>
-      </c>
-      <c r="H4" s="19">
-        <f>G4*(1+Calculateur!$E$6/100)</f>
-        <v>21.361249999999998</v>
-      </c>
-      <c r="I4" s="19">
-        <f>H4*E4*(1-Calculateur!$E$8/100)</f>
-        <v>64.083749999999995</v>
-      </c>
-      <c r="J4" s="19">
-        <f>I4*Calculateur!$E$7/100</f>
-        <v>13.457587499999999</v>
-      </c>
-      <c r="K4" s="19">
-        <f t="shared" si="1"/>
-        <v>77.541337499999997</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="17">
-        <v>250</v>
-      </c>
-      <c r="B5" s="17">
-        <v>8</v>
-      </c>
-      <c r="C5" s="17" t="s">
+      <c r="G12" s="27">
+        <f>B12*Calculateur!$B$6*Calculateur!$B$12*(C12/Calculateur!$B$13)*IF(D12="1 IA",1,IF(D12="2 IA",1.55,IF(D12="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>13.8125</v>
+      </c>
+      <c r="H12" s="27">
+        <f t="shared" ref="H12:H19" si="2">G12+IF(E12="Aucun",0,IF(E12="Synthèse courte",2,6))</f>
+        <v>15.8125</v>
+      </c>
+      <c r="I12" s="27">
+        <f>H12*(1+Calculateur!$E$6/100)</f>
+        <v>18.184374999999999</v>
+      </c>
+      <c r="J12" s="17">
+        <f>I12*F12*(1-Calculateur!$E$8/100)</f>
+        <v>54.553124999999994</v>
+      </c>
+      <c r="K12" s="17">
+        <f>J12*Calculateur!$E$7/100</f>
+        <v>11.456156249999999</v>
+      </c>
+      <c r="L12" s="28">
+        <f t="shared" ref="L12:L19" si="3">J12+K12</f>
+        <v>66.009281249999987</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" s="44" t="s">
+        <v>105</v>
+      </c>
+      <c r="B13" s="45">
+        <v>125</v>
+      </c>
+      <c r="C13" s="45">
+        <v>15</v>
+      </c>
+      <c r="D13" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="E13" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="E5" s="18">
+      <c r="F13" s="53">
         <v>3</v>
       </c>
-      <c r="F5" s="19">
-        <f>A5*Calculateur!$B$6*Calculateur!$B$12*(B5/Calculateur!$B$13)*IF(C5="1 IA",1,IF(C5="2 IA",1.55,IF(C5="2 IA + confrontation ciblée",1.9,2.35)))</f>
-        <v>27.625</v>
-      </c>
-      <c r="G5" s="19">
-        <f>F5+IF(D5="Aucun",0,IF(D5="Synthèse courte",2,6))</f>
-        <v>29.625</v>
-      </c>
-      <c r="H5" s="19">
-        <f>G5*(1+Calculateur!$E$6/100)</f>
-        <v>34.068749999999994</v>
-      </c>
-      <c r="I5" s="19">
-        <f>H5*E5*(1-Calculateur!$E$8/100)</f>
-        <v>102.20624999999998</v>
-      </c>
-      <c r="J5" s="19">
-        <f>I5*Calculateur!$E$7/100</f>
-        <v>21.463312499999997</v>
-      </c>
-      <c r="K5" s="19">
-        <f>I5+J5</f>
-        <v>123.66956249999998</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="A6" s="17">
-        <v>150</v>
-      </c>
-      <c r="B6" s="17">
+      <c r="G13" s="46">
+        <f>B13*Calculateur!$B$6*Calculateur!$B$12*(C13/Calculateur!$B$13)*IF(D13="1 IA",1,IF(D13="2 IA",1.55,IF(D13="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>25.8984375</v>
+      </c>
+      <c r="H13" s="46">
+        <f>G13+IF(E13="Aucun",0,IF(E13="Synthèse courte",2,6))</f>
+        <v>27.8984375</v>
+      </c>
+      <c r="I13" s="46">
+        <f>H13*(1+Calculateur!$E$6/100)</f>
+        <v>32.083203124999997</v>
+      </c>
+      <c r="J13" s="47">
+        <f>I13*F13*(1-Calculateur!$E$8/100)</f>
+        <v>96.249609374999991</v>
+      </c>
+      <c r="K13" s="47">
+        <f>J13*Calculateur!$E$7/100</f>
+        <v>20.21241796875</v>
+      </c>
+      <c r="L13" s="48">
+        <f>J13+K13</f>
+        <v>116.46202734374999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" s="41" t="s">
+        <v>105</v>
+      </c>
+      <c r="B14" s="40">
+        <v>125</v>
+      </c>
+      <c r="C14" s="40">
         <v>15</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="D14" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="E14" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="18">
+      <c r="F14" s="52">
         <v>4</v>
       </c>
-      <c r="F6" s="19">
-        <f>A6*Calculateur!$B$6*Calculateur!$B$12*(B6/Calculateur!$B$13)*IF(C6="1 IA",1,IF(C6="2 IA",1.55,IF(C6="2 IA + confrontation ciblée",1.9,2.35)))</f>
-        <v>31.078125</v>
-      </c>
-      <c r="G6" s="19">
-        <f t="shared" si="0"/>
-        <v>37.078125</v>
-      </c>
-      <c r="H6" s="19">
-        <f>G6*(1+Calculateur!$E$6/100)</f>
-        <v>42.639843749999997</v>
-      </c>
-      <c r="I6" s="19">
-        <f>H6*E6*(1-Calculateur!$E$8/100)</f>
-        <v>170.55937499999999</v>
-      </c>
-      <c r="J6" s="19">
-        <f>I6*Calculateur!$E$7/100</f>
-        <v>35.817468749999996</v>
-      </c>
-      <c r="K6" s="19">
-        <f t="shared" si="1"/>
-        <v>206.37684374999998</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
-      <c r="A7" s="17">
-        <v>150</v>
-      </c>
-      <c r="B7" s="17">
+      <c r="G14" s="27">
+        <f>B14*Calculateur!$B$6*Calculateur!$B$12*(C14/Calculateur!$B$13)*IF(D14="1 IA",1,IF(D14="2 IA",1.55,IF(D14="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>25.8984375</v>
+      </c>
+      <c r="H14" s="27">
+        <f t="shared" si="2"/>
+        <v>31.8984375</v>
+      </c>
+      <c r="I14" s="27">
+        <f>H14*(1+Calculateur!$E$6/100)</f>
+        <v>36.683203124999999</v>
+      </c>
+      <c r="J14" s="17">
+        <f>I14*F14*(1-Calculateur!$E$8/100)</f>
+        <v>146.73281249999999</v>
+      </c>
+      <c r="K14" s="17">
+        <f>J14*Calculateur!$E$7/100</f>
+        <v>30.813890624999999</v>
+      </c>
+      <c r="L14" s="28">
+        <f t="shared" si="3"/>
+        <v>177.54670312499999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="B15" s="40">
+        <v>200</v>
+      </c>
+      <c r="C15" s="40">
         <v>30</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="D15" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="E15" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="18">
+      <c r="F15" s="52">
         <v>4</v>
       </c>
-      <c r="F7" s="19">
-        <f>A7*Calculateur!$B$6*Calculateur!$B$12*(B7/Calculateur!$B$13)*IF(C7="1 IA",1,IF(C7="2 IA",1.55,IF(C7="2 IA + confrontation ciblée",1.9,2.35)))</f>
-        <v>62.15625</v>
-      </c>
-      <c r="G7" s="19">
-        <f t="shared" si="0"/>
-        <v>68.15625</v>
-      </c>
-      <c r="H7" s="19">
-        <f>G7*(1+Calculateur!$E$6/100)</f>
-        <v>78.379687499999989</v>
-      </c>
-      <c r="I7" s="19">
-        <f>H7*E7*(1-Calculateur!$E$8/100)</f>
-        <v>313.51874999999995</v>
-      </c>
-      <c r="J7" s="19">
-        <f>I7*Calculateur!$E$7/100</f>
-        <v>65.838937499999986</v>
-      </c>
-      <c r="K7" s="19">
-        <f t="shared" si="1"/>
-        <v>379.35768749999994</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
-      <c r="A8" s="17">
-        <v>150</v>
-      </c>
-      <c r="B8" s="17">
+      <c r="G15" s="27">
+        <f>B15*Calculateur!$B$6*Calculateur!$B$12*(C15/Calculateur!$B$13)*IF(D15="1 IA",1,IF(D15="2 IA",1.55,IF(D15="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>82.874999999999986</v>
+      </c>
+      <c r="H15" s="27">
+        <f t="shared" si="2"/>
+        <v>88.874999999999986</v>
+      </c>
+      <c r="I15" s="27">
+        <f>H15*(1+Calculateur!$E$6/100)</f>
+        <v>102.20624999999997</v>
+      </c>
+      <c r="J15" s="17">
+        <f>I15*F15*(1-Calculateur!$E$8/100)</f>
+        <v>408.82499999999987</v>
+      </c>
+      <c r="K15" s="17">
+        <f>J15*Calculateur!$E$7/100</f>
+        <v>85.853249999999974</v>
+      </c>
+      <c r="L15" s="28">
+        <f t="shared" si="3"/>
+        <v>494.67824999999982</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="B16" s="40">
+        <v>200</v>
+      </c>
+      <c r="C16" s="40">
         <v>30</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="D16" s="40" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="E16" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="18">
+      <c r="F16" s="52">
         <v>4</v>
       </c>
-      <c r="F8" s="19">
-        <f>A8*Calculateur!$B$6*Calculateur!$B$12*(B8/Calculateur!$B$13)*IF(C8="1 IA",1,IF(C8="2 IA",1.55,IF(C8="2 IA + confrontation ciblée",1.9,2.35)))</f>
-        <v>96.342187500000009</v>
-      </c>
-      <c r="G8" s="19">
-        <f t="shared" si="0"/>
-        <v>102.34218750000001</v>
-      </c>
-      <c r="H8" s="19">
-        <f>G8*(1+Calculateur!$E$6/100)</f>
-        <v>117.693515625</v>
-      </c>
-      <c r="I8" s="19">
-        <f>H8*E8*(1-Calculateur!$E$8/100)</f>
-        <v>470.77406250000001</v>
-      </c>
-      <c r="J8" s="19">
-        <f>I8*Calculateur!$E$7/100</f>
-        <v>98.862553124999991</v>
-      </c>
-      <c r="K8" s="19">
-        <f t="shared" si="1"/>
-        <v>569.63661562499999</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
-      <c r="A9" s="17">
-        <v>150</v>
-      </c>
-      <c r="B9" s="17">
+      <c r="G16" s="27">
+        <f>B16*Calculateur!$B$6*Calculateur!$B$12*(C16/Calculateur!$B$13)*IF(D16="1 IA",1,IF(D16="2 IA",1.55,IF(D16="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>128.45624999999998</v>
+      </c>
+      <c r="H16" s="27">
+        <f t="shared" si="2"/>
+        <v>134.45624999999998</v>
+      </c>
+      <c r="I16" s="27">
+        <f>H16*(1+Calculateur!$E$6/100)</f>
+        <v>154.62468749999996</v>
+      </c>
+      <c r="J16" s="17">
+        <f>I16*F16*(1-Calculateur!$E$8/100)</f>
+        <v>618.49874999999986</v>
+      </c>
+      <c r="K16" s="17">
+        <f>J16*Calculateur!$E$7/100</f>
+        <v>129.88473749999997</v>
+      </c>
+      <c r="L16" s="28">
+        <f t="shared" si="3"/>
+        <v>748.38348749999977</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="B17" s="40">
+        <v>200</v>
+      </c>
+      <c r="C17" s="40">
         <v>30</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="D17" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="E17" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="18">
+      <c r="F17" s="52">
         <v>4</v>
       </c>
-      <c r="F9" s="19">
-        <f>A9*Calculateur!$B$6*Calculateur!$B$12*(B9/Calculateur!$B$13)*IF(C9="1 IA",1,IF(C9="2 IA",1.55,IF(C9="2 IA + confrontation ciblée",1.9,2.35)))</f>
-        <v>118.096875</v>
-      </c>
-      <c r="G9" s="19">
-        <f t="shared" si="0"/>
-        <v>124.096875</v>
-      </c>
-      <c r="H9" s="19">
-        <f>G9*(1+Calculateur!$E$6/100)</f>
-        <v>142.71140624999998</v>
-      </c>
-      <c r="I9" s="19">
-        <f>H9*E9*(1-Calculateur!$E$8/100)</f>
-        <v>570.84562499999993</v>
-      </c>
-      <c r="J9" s="19">
-        <f>I9*Calculateur!$E$7/100</f>
-        <v>119.87758124999999</v>
-      </c>
-      <c r="K9" s="19">
-        <f t="shared" si="1"/>
-        <v>690.72320624999998</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
-      <c r="A10" s="17">
-        <v>150</v>
-      </c>
-      <c r="B10" s="17">
+      <c r="G17" s="27">
+        <f>B17*Calculateur!$B$6*Calculateur!$B$12*(C17/Calculateur!$B$13)*IF(D17="1 IA",1,IF(D17="2 IA",1.55,IF(D17="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>157.46249999999998</v>
+      </c>
+      <c r="H17" s="27">
+        <f t="shared" si="2"/>
+        <v>163.46249999999998</v>
+      </c>
+      <c r="I17" s="27">
+        <f>H17*(1+Calculateur!$E$6/100)</f>
+        <v>187.98187499999995</v>
+      </c>
+      <c r="J17" s="17">
+        <f>I17*F17*(1-Calculateur!$E$8/100)</f>
+        <v>751.92749999999978</v>
+      </c>
+      <c r="K17" s="17">
+        <f>J17*Calculateur!$E$7/100</f>
+        <v>157.90477499999994</v>
+      </c>
+      <c r="L17" s="28">
+        <f t="shared" si="3"/>
+        <v>909.83227499999975</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" s="39" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" s="40">
+        <v>200</v>
+      </c>
+      <c r="C18" s="40">
         <v>30</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="D18" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="E18" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="18">
+      <c r="F18" s="52">
         <v>4</v>
       </c>
-      <c r="F10" s="19">
-        <f>A10*Calculateur!$B$6*Calculateur!$B$12*(B10/Calculateur!$B$13)*IF(C10="1 IA",1,IF(C10="2 IA",1.55,IF(C10="2 IA + confrontation ciblée",1.9,2.35)))</f>
-        <v>146.06718750000002</v>
-      </c>
-      <c r="G10" s="19">
-        <f t="shared" si="0"/>
-        <v>152.06718750000002</v>
-      </c>
-      <c r="H10" s="19">
-        <f>G10*(1+Calculateur!$E$6/100)</f>
-        <v>174.87726562500001</v>
-      </c>
-      <c r="I10" s="19">
-        <f>H10*E10*(1-Calculateur!$E$8/100)</f>
-        <v>699.50906250000003</v>
-      </c>
-      <c r="J10" s="19">
-        <f>I10*Calculateur!$E$7/100</f>
-        <v>146.89690312499999</v>
-      </c>
-      <c r="K10" s="19">
-        <f t="shared" si="1"/>
-        <v>846.40596562500002</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
-      <c r="A11" s="17">
-        <v>250</v>
-      </c>
-      <c r="B11" s="17">
+      <c r="G18" s="27">
+        <f>B18*Calculateur!$B$6*Calculateur!$B$12*(C18/Calculateur!$B$13)*IF(D18="1 IA",1,IF(D18="2 IA",1.55,IF(D18="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>194.75624999999997</v>
+      </c>
+      <c r="H18" s="27">
+        <f t="shared" si="2"/>
+        <v>200.75624999999997</v>
+      </c>
+      <c r="I18" s="27">
+        <f>H18*(1+Calculateur!$E$6/100)</f>
+        <v>230.86968749999994</v>
+      </c>
+      <c r="J18" s="17">
+        <f>I18*F18*(1-Calculateur!$E$8/100)</f>
+        <v>923.47874999999976</v>
+      </c>
+      <c r="K18" s="17">
+        <f>J18*Calculateur!$E$7/100</f>
+        <v>193.93053749999996</v>
+      </c>
+      <c r="L18" s="28">
+        <f t="shared" si="3"/>
+        <v>1117.4092874999997</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="15" thickBot="1">
+      <c r="A19" s="42" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19" s="43">
+        <v>300</v>
+      </c>
+      <c r="C19" s="43">
         <v>30</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="D19" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="E19" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="18">
-        <v>5</v>
-      </c>
-      <c r="F11" s="19">
-        <f>A11*Calculateur!$B$6*Calculateur!$B$12*(B11/Calculateur!$B$13)*IF(C11="1 IA",1,IF(C11="2 IA",1.55,IF(C11="2 IA + confrontation ciblée",1.9,2.35)))</f>
-        <v>243.4453125</v>
-      </c>
-      <c r="G11" s="19">
-        <f t="shared" si="0"/>
-        <v>249.4453125</v>
-      </c>
-      <c r="H11" s="19">
-        <f>G11*(1+Calculateur!$E$6/100)</f>
-        <v>286.86210937499999</v>
-      </c>
-      <c r="I11" s="19">
-        <f>H11*E11*(1-Calculateur!$E$8/100)</f>
-        <v>1434.310546875</v>
-      </c>
-      <c r="J11" s="19">
-        <f>I11*Calculateur!$E$7/100</f>
-        <v>301.20521484375001</v>
-      </c>
-      <c r="K11" s="19">
-        <f t="shared" si="1"/>
-        <v>1735.5157617187501</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
-    </row>
-    <row r="13" spans="1:11">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-    </row>
-    <row r="14" spans="1:11">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
-    </row>
-    <row r="15" spans="1:11">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
-      <c r="K15" s="1"/>
-    </row>
-    <row r="16" spans="1:11">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-    </row>
-    <row r="17" spans="1:11">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
-    </row>
-    <row r="18" spans="1:11">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
-    </row>
-    <row r="19" spans="1:11">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-    </row>
-    <row r="20" spans="1:11">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
+      <c r="F19" s="54">
+        <v>4</v>
+      </c>
+      <c r="G19" s="34">
+        <f>B19*Calculateur!$B$6*Calculateur!$B$12*(C19/Calculateur!$B$13)*IF(D19="1 IA",1,IF(D19="2 IA",1.55,IF(D19="2 IA + confrontation ciblée",1.9,2.35)))</f>
+        <v>292.13437500000003</v>
+      </c>
+      <c r="H19" s="34">
+        <f t="shared" si="2"/>
+        <v>298.13437500000003</v>
+      </c>
+      <c r="I19" s="34">
+        <f>H19*(1+Calculateur!$E$6/100)</f>
+        <v>342.85453125000004</v>
+      </c>
+      <c r="J19" s="35">
+        <f>I19*F19*(1-Calculateur!$E$8/100)</f>
+        <v>1371.4181250000001</v>
+      </c>
+      <c r="K19" s="35">
+        <f>J19*Calculateur!$E$7/100</f>
+        <v>287.99780625000005</v>
+      </c>
+      <c r="L19" s="36">
+        <f t="shared" si="3"/>
+        <v>1659.4159312500001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
+      <c r="A20" s="19"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
-    </row>
-    <row r="21" spans="1:11">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
+      <c r="L20" s="1"/>
+    </row>
+    <row r="21" spans="1:12">
+      <c r="A21" s="19"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="19"/>
+      <c r="H21" s="19"/>
+      <c r="I21" s="19"/>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
-    </row>
-    <row r="22" spans="1:11">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
+      <c r="L21" s="1"/>
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22" s="19"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="19"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
-    </row>
-    <row r="23" spans="1:11">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
+      <c r="L22" s="1"/>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" s="19"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="19"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
-    </row>
-    <row r="24" spans="1:11">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
+      <c r="L23" s="1"/>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" s="19"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="19"/>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
-    </row>
-    <row r="25" spans="1:11">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
+      <c r="L24" s="1"/>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" s="19"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="19"/>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
-    </row>
-    <row r="26" spans="1:11">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
+      <c r="L25" s="1"/>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26" s="19"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="19"/>
+      <c r="H26" s="19"/>
+      <c r="I26" s="19"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
-    </row>
-    <row r="27" spans="1:11">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
-      <c r="I27" s="1"/>
+      <c r="L26" s="1"/>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="A27" s="19"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="19"/>
+      <c r="H27" s="19"/>
+      <c r="I27" s="19"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
-    </row>
-    <row r="28" spans="1:11">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
+      <c r="L27" s="1"/>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" s="19"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="19"/>
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
-    </row>
-    <row r="29" spans="1:11">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
+      <c r="L28" s="1"/>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="A29" s="19"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
+      <c r="G29" s="19"/>
+      <c r="H29" s="19"/>
+      <c r="I29" s="19"/>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
-    </row>
-    <row r="30" spans="1:11">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
+      <c r="L29" s="1"/>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" s="19"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="19"/>
+      <c r="G30" s="19"/>
+      <c r="H30" s="19"/>
+      <c r="I30" s="19"/>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" s="19"/>
+      <c r="B31" s="19"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="19"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="A32" s="19"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="19"/>
+      <c r="G32" s="19"/>
+      <c r="H32" s="19"/>
+      <c r="I32" s="19"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+    </row>
+    <row r="33" spans="1:12">
+      <c r="A33" s="19"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="19"/>
+      <c r="H33" s="19"/>
+      <c r="I33" s="19"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+    </row>
+    <row r="34" spans="1:12">
+      <c r="A34" s="19"/>
+      <c r="B34" s="19"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="19"/>
+      <c r="F34" s="19"/>
+      <c r="G34" s="19"/>
+      <c r="H34" s="19"/>
+      <c r="I34" s="19"/>
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+    </row>
+    <row r="35" spans="1:12">
+      <c r="A35" s="19"/>
+      <c r="B35" s="19"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="19"/>
+      <c r="E35" s="19"/>
+      <c r="F35" s="19"/>
+      <c r="G35" s="19"/>
+      <c r="H35" s="19"/>
+      <c r="I35" s="19"/>
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
+      <c r="L35" s="1"/>
+    </row>
+    <row r="36" spans="1:12">
+      <c r="A36" s="19"/>
+      <c r="B36" s="19"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="19"/>
+      <c r="F36" s="19"/>
+      <c r="G36" s="19"/>
+      <c r="H36" s="19"/>
+      <c r="I36" s="19"/>
+      <c r="J36" s="1"/>
+      <c r="K36" s="1"/>
+      <c r="L36" s="1"/>
+    </row>
+    <row r="37" spans="1:12">
+      <c r="A37" s="19"/>
+      <c r="B37" s="19"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="19"/>
+      <c r="E37" s="19"/>
+      <c r="F37" s="19"/>
+      <c r="G37" s="19"/>
+      <c r="H37" s="19"/>
+      <c r="I37" s="19"/>
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
+      <c r="L37" s="1"/>
+    </row>
+    <row r="38" spans="1:12">
+      <c r="A38" s="19"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="19"/>
+      <c r="H38" s="19"/>
+      <c r="I38" s="19"/>
+      <c r="J38" s="1"/>
+      <c r="K38" s="1"/>
+      <c r="L38" s="1"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:K11">
+  <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="J2:L19">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="min"/>
@@ -3799,7 +4464,7 @@
               <x14:axisColor auto="1"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>I2:K11</xm:sqref>
+          <xm:sqref>J2:L19</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>